<commit_message>
minor change topic 2
</commit_message>
<xml_diff>
--- a/topic_2_img/Topic 2 Sol.xlsx
+++ b/topic_2_img/Topic 2 Sol.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Data/Github/lecture_financial_statements_analysis/topic_2_img/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CBB5505-16DA-A942-BDCA-6068B6287A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A805BADB-298C-4C4F-ACCF-D1AF02E91AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-35560" yWindow="2040" windowWidth="36060" windowHeight="20640" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_loan" sheetId="1" r:id="rId1"/>
@@ -461,12 +461,6 @@
   </cellStyleXfs>
   <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -498,6 +492,12 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -771,7 +771,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
@@ -779,7 +779,7 @@
       <c r="B4" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="2">
         <v>1000000</v>
       </c>
     </row>
@@ -787,222 +787,222 @@
       <c r="B5" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="3">
         <v>0.05</v>
       </c>
     </row>
     <row r="7" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="9" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="I9" s="2" t="s">
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="I9" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="J9" s="2"/>
-      <c r="L9" s="2" t="s">
+      <c r="J9" s="32"/>
+      <c r="L9" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="M9" s="2"/>
+      <c r="M9" s="32"/>
     </row>
     <row r="10" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G10" s="9"/>
-      <c r="I10" s="10" t="s">
+      <c r="G10" s="7"/>
+      <c r="I10" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="J10" s="11"/>
-      <c r="L10" s="7" t="s">
+      <c r="J10" s="9"/>
+      <c r="L10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M10" s="9"/>
+      <c r="M10" s="7"/>
     </row>
     <row r="11" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D11" s="10"/>
-      <c r="E11" s="4"/>
-      <c r="G11" s="9"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="11"/>
-      <c r="L11" s="10" t="s">
+      <c r="D11" s="8"/>
+      <c r="E11" s="2"/>
+      <c r="G11" s="7"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="9"/>
+      <c r="L11" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="M11" s="11">
+      <c r="M11" s="9">
         <v>1000000</v>
       </c>
     </row>
     <row r="12" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="2">
         <v>1000000</v>
       </c>
-      <c r="G12" s="9"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="11"/>
-      <c r="L12" s="10"/>
-      <c r="M12" s="11"/>
+      <c r="G12" s="7"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="9"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="9"/>
     </row>
     <row r="13" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D13" s="10"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="8" t="s">
+      <c r="D13" s="8"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="9"/>
-      <c r="I13" s="7" t="s">
+      <c r="G13" s="7"/>
+      <c r="I13" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="11"/>
-      <c r="L13" s="7" t="s">
+      <c r="J13" s="9"/>
+      <c r="L13" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="M13" s="11"/>
+      <c r="M13" s="9"/>
     </row>
     <row r="14" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D14" s="10"/>
-      <c r="E14" s="4"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="2"/>
       <c r="F14" t="s">
         <v>16</v>
       </c>
-      <c r="G14" s="11">
+      <c r="G14" s="9">
         <v>1000000</v>
       </c>
-      <c r="I14" s="10"/>
-      <c r="J14" s="11"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="11"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="9"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="9"/>
     </row>
     <row r="15" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D15" s="12"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="15"/>
-      <c r="I15" s="16" t="s">
+      <c r="D15" s="10"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="13"/>
+      <c r="I15" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="J15" s="17"/>
-      <c r="L15" s="12"/>
-      <c r="M15" s="17"/>
+      <c r="J15" s="15"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="15"/>
     </row>
     <row r="18" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="I20" s="2" t="s">
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+      <c r="I20" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="J20" s="2"/>
-      <c r="L20" s="2" t="s">
+      <c r="J20" s="32"/>
+      <c r="L20" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="M20" s="2"/>
+      <c r="M20" s="32"/>
     </row>
     <row r="21" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G21" s="9"/>
-      <c r="I21" s="7" t="s">
+      <c r="G21" s="7"/>
+      <c r="I21" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="J21" s="11"/>
-      <c r="L21" s="7" t="s">
+      <c r="J21" s="9"/>
+      <c r="L21" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M21" s="9"/>
+      <c r="M21" s="7"/>
     </row>
     <row r="22" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D22" s="10"/>
-      <c r="E22" s="4"/>
-      <c r="G22" s="9"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="11"/>
-      <c r="L22" s="10"/>
-      <c r="M22" s="11"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="2"/>
+      <c r="G22" s="7"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="9"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="9"/>
     </row>
     <row r="23" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D23" s="10"/>
-      <c r="E23" s="4"/>
-      <c r="G23" s="9"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="11"/>
-      <c r="L23" s="10"/>
-      <c r="M23" s="11"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="2"/>
+      <c r="G23" s="7"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="9"/>
+      <c r="L23" s="8"/>
+      <c r="M23" s="9"/>
     </row>
     <row r="24" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D24" s="10"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="8" t="s">
+      <c r="D24" s="8"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G24" s="9"/>
-      <c r="I24" s="7" t="s">
+      <c r="G24" s="7"/>
+      <c r="I24" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J24" s="11"/>
-      <c r="L24" s="7" t="s">
+      <c r="J24" s="9"/>
+      <c r="L24" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="M24" s="11"/>
+      <c r="M24" s="9"/>
     </row>
     <row r="25" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D25" s="10"/>
-      <c r="E25" s="4"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="2"/>
       <c r="F25" t="s">
         <v>19</v>
       </c>
-      <c r="G25" s="11">
+      <c r="G25" s="9">
         <f>+C5*C4</f>
         <v>50000</v>
       </c>
-      <c r="I25" s="10" t="s">
+      <c r="I25" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="J25" s="11">
+      <c r="J25" s="9">
         <f>+-G25</f>
         <v>-50000</v>
       </c>
-      <c r="L25" s="10"/>
-      <c r="M25" s="11"/>
+      <c r="L25" s="8"/>
+      <c r="M25" s="9"/>
     </row>
     <row r="26" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D26" s="12"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="15"/>
-      <c r="I26" s="16" t="s">
+      <c r="D26" s="10"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="13"/>
+      <c r="I26" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="J26" s="17">
+      <c r="J26" s="15">
         <f>SUM(J21:J25)</f>
         <v>-50000</v>
       </c>
-      <c r="L26" s="12"/>
-      <c r="M26" s="17"/>
+      <c r="L26" s="10"/>
+      <c r="M26" s="15"/>
     </row>
     <row r="29" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B29" t="s">
@@ -1010,799 +1010,799 @@
       </c>
     </row>
     <row r="30" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15"/>
-    <row r="32" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15"/>
+    <row r="32" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
       <c r="B32" t="s">
         <v>1</v>
       </c>
-      <c r="C32" s="4">
+      <c r="C32" s="2">
         <v>1000000</v>
       </c>
     </row>
-    <row r="33" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
       <c r="B33" t="s">
         <v>2</v>
       </c>
-      <c r="C33" s="5">
+      <c r="C33" s="3">
         <v>0.05</v>
       </c>
     </row>
-    <row r="34" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15"/>
-    <row r="35" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="B35" s="6" t="s">
+    <row r="34" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15"/>
+    <row r="35" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="B35" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="36" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15"/>
-    <row r="37" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D37" s="1" t="s">
+    <row r="36" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15"/>
+    <row r="37" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D37" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="E37" s="1"/>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="I37" s="1" t="s">
+      <c r="E37" s="33"/>
+      <c r="F37" s="33"/>
+      <c r="G37" s="33"/>
+      <c r="I37" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="J37" s="1"/>
-      <c r="L37" s="1" t="s">
+      <c r="J37" s="33"/>
+      <c r="L37" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="M37" s="1"/>
-    </row>
-    <row r="38" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D38" s="18" t="s">
+      <c r="M37" s="33"/>
+    </row>
+    <row r="38" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D38" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="E38" s="19"/>
-      <c r="F38" s="20" t="s">
+      <c r="E38" s="17"/>
+      <c r="F38" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="G38" s="21"/>
-      <c r="I38" s="22" t="s">
+      <c r="G38" s="19"/>
+      <c r="I38" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="J38" s="23"/>
-      <c r="L38" s="18" t="s">
+      <c r="J38" s="21"/>
+      <c r="L38" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="M38" s="21"/>
-    </row>
-    <row r="39" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D39" s="22"/>
-      <c r="E39" s="24"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="23"/>
-      <c r="I39" s="22"/>
-      <c r="J39" s="23"/>
-      <c r="L39" s="22"/>
-      <c r="M39" s="23"/>
-    </row>
-    <row r="40" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D40" s="22"/>
-      <c r="E40" s="24"/>
-      <c r="F40" s="19"/>
-      <c r="G40" s="21"/>
-      <c r="I40" s="22"/>
-      <c r="J40" s="23"/>
-      <c r="L40" s="22"/>
-      <c r="M40" s="23"/>
-    </row>
-    <row r="41" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D41" s="22"/>
-      <c r="E41" s="24"/>
-      <c r="F41" s="20" t="s">
+      <c r="M38" s="19"/>
+    </row>
+    <row r="39" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D39" s="20"/>
+      <c r="E39" s="22"/>
+      <c r="F39" s="17"/>
+      <c r="G39" s="21"/>
+      <c r="I39" s="20"/>
+      <c r="J39" s="21"/>
+      <c r="L39" s="20"/>
+      <c r="M39" s="21"/>
+    </row>
+    <row r="40" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D40" s="20"/>
+      <c r="E40" s="22"/>
+      <c r="F40" s="17"/>
+      <c r="G40" s="19"/>
+      <c r="I40" s="20"/>
+      <c r="J40" s="21"/>
+      <c r="L40" s="20"/>
+      <c r="M40" s="21"/>
+    </row>
+    <row r="41" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D41" s="20"/>
+      <c r="E41" s="22"/>
+      <c r="F41" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G41" s="21"/>
-      <c r="I41" s="18" t="s">
+      <c r="G41" s="19"/>
+      <c r="I41" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="J41" s="23"/>
-      <c r="L41" s="18" t="s">
+      <c r="J41" s="21"/>
+      <c r="L41" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="M41" s="23"/>
-    </row>
-    <row r="42" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D42" s="22"/>
-      <c r="E42" s="24"/>
-      <c r="F42" s="19" t="s">
+      <c r="M41" s="21"/>
+    </row>
+    <row r="42" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D42" s="20"/>
+      <c r="E42" s="22"/>
+      <c r="F42" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="G42" s="23">
+      <c r="G42" s="21">
         <v>1000000</v>
       </c>
-      <c r="I42" s="22" t="s">
+      <c r="I42" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="J42" s="23">
+      <c r="J42" s="21">
         <f>-G43</f>
         <v>-50000</v>
       </c>
-      <c r="L42" s="22"/>
-      <c r="M42" s="23"/>
-    </row>
-    <row r="43" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D43" s="25"/>
-      <c r="E43" s="26"/>
-      <c r="F43" s="27" t="s">
+      <c r="L42" s="20"/>
+      <c r="M42" s="21"/>
+    </row>
+    <row r="43" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D43" s="23"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="G43" s="28">
+      <c r="G43" s="26">
         <f>C4*C5</f>
         <v>50000</v>
       </c>
-      <c r="I43" s="29" t="s">
+      <c r="I43" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="J43" s="28">
+      <c r="J43" s="26">
         <f>J42</f>
         <v>-50000</v>
       </c>
-      <c r="L43" s="25"/>
-      <c r="M43" s="28"/>
-    </row>
-    <row r="44" spans="2:13" ht="13" collapsed="1" x14ac:dyDescent="0.15">
-      <c r="B44" s="6" t="s">
+      <c r="L43" s="23"/>
+      <c r="M43" s="26"/>
+    </row>
+    <row r="44" spans="2:13" ht="13" x14ac:dyDescent="0.15">
+      <c r="B44" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="45" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D45" s="2" t="s">
+      <c r="D45" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-      <c r="I45" s="2" t="s">
+      <c r="E45" s="32"/>
+      <c r="F45" s="32"/>
+      <c r="G45" s="32"/>
+      <c r="I45" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="J45" s="2"/>
-      <c r="L45" s="2" t="s">
+      <c r="J45" s="32"/>
+      <c r="L45" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="M45" s="2"/>
+      <c r="M45" s="32"/>
     </row>
     <row r="46" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D46" s="7" t="s">
+      <c r="D46" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F46" s="8" t="s">
+      <c r="F46" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G46" s="9"/>
-      <c r="I46" s="10" t="s">
+      <c r="G46" s="7"/>
+      <c r="I46" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="J46" s="11"/>
-      <c r="L46" s="7" t="s">
+      <c r="J46" s="9"/>
+      <c r="L46" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M46" s="9"/>
+      <c r="M46" s="7"/>
     </row>
     <row r="47" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D47" s="10" t="s">
+      <c r="D47" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E47" s="4">
+      <c r="E47" s="2">
         <f>+-(G42+G43)</f>
         <v>-1050000</v>
       </c>
-      <c r="G47" s="11"/>
-      <c r="I47" s="10"/>
-      <c r="J47" s="11"/>
-      <c r="L47" s="10"/>
-      <c r="M47" s="11"/>
+      <c r="G47" s="9"/>
+      <c r="I47" s="8"/>
+      <c r="J47" s="9"/>
+      <c r="L47" s="8"/>
+      <c r="M47" s="9"/>
     </row>
     <row r="48" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D48" s="10"/>
-      <c r="E48" s="4"/>
-      <c r="G48" s="9"/>
-      <c r="I48" s="10"/>
-      <c r="J48" s="11"/>
-      <c r="L48" s="10"/>
-      <c r="M48" s="11"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="2"/>
+      <c r="G48" s="7"/>
+      <c r="I48" s="8"/>
+      <c r="J48" s="9"/>
+      <c r="L48" s="8"/>
+      <c r="M48" s="9"/>
     </row>
     <row r="49" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D49" s="10"/>
-      <c r="E49" s="4"/>
-      <c r="F49" s="8" t="s">
+      <c r="D49" s="8"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G49" s="9"/>
-      <c r="I49" s="7" t="s">
+      <c r="G49" s="7"/>
+      <c r="I49" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J49" s="11"/>
-      <c r="L49" s="7" t="s">
+      <c r="J49" s="9"/>
+      <c r="L49" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="M49" s="11"/>
+      <c r="M49" s="9"/>
     </row>
     <row r="50" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D50" s="10"/>
-      <c r="E50" s="4"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="2"/>
       <c r="F50" t="s">
         <v>24</v>
       </c>
-      <c r="G50" s="11">
+      <c r="G50" s="9">
         <f>-G42</f>
         <v>-1000000</v>
       </c>
-      <c r="I50" s="10"/>
-      <c r="J50" s="11"/>
-      <c r="L50" s="10" t="s">
+      <c r="I50" s="8"/>
+      <c r="J50" s="9"/>
+      <c r="L50" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="M50" s="11">
+      <c r="M50" s="9">
         <f>+E47</f>
         <v>-1050000</v>
       </c>
     </row>
     <row r="51" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D51" s="12"/>
-      <c r="E51" s="13"/>
-      <c r="F51" s="14" t="s">
+      <c r="D51" s="10"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="G51" s="17">
+      <c r="G51" s="15">
         <f>-G43</f>
         <v>-50000</v>
       </c>
-      <c r="I51" s="16" t="s">
+      <c r="I51" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="J51" s="17"/>
-      <c r="L51" s="12"/>
-      <c r="M51" s="17"/>
+      <c r="J51" s="15"/>
+      <c r="L51" s="10"/>
+      <c r="M51" s="15"/>
     </row>
     <row r="54" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="B54" s="3" t="s">
+      <c r="B54" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="55" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15"/>
-    <row r="56" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
+    <row r="55" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15"/>
+    <row r="56" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
       <c r="B56" t="s">
         <v>1</v>
       </c>
-      <c r="C56" s="4">
+      <c r="C56" s="2">
         <v>1000000</v>
       </c>
     </row>
-    <row r="57" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
+    <row r="57" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
       <c r="B57" t="s">
         <v>2</v>
       </c>
-      <c r="C57" s="5">
+      <c r="C57" s="3">
         <v>0.05</v>
       </c>
-      <c r="D57" s="5">
+      <c r="D57" s="3">
         <v>0.1</v>
       </c>
     </row>
-    <row r="58" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15"/>
-    <row r="59" spans="2:13" ht="15" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="B59" s="6" t="s">
+    <row r="58" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15"/>
+    <row r="59" spans="2:13" ht="15" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="B59" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="60" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15"/>
-    <row r="61" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D61" s="1" t="s">
+    <row r="60" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15"/>
+    <row r="61" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D61" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="E61" s="1"/>
-      <c r="F61" s="1"/>
-      <c r="G61" s="1"/>
-      <c r="I61" s="1" t="s">
+      <c r="E61" s="33"/>
+      <c r="F61" s="33"/>
+      <c r="G61" s="33"/>
+      <c r="I61" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="J61" s="1"/>
-      <c r="L61" s="1" t="s">
+      <c r="J61" s="33"/>
+      <c r="L61" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="M61" s="1"/>
-    </row>
-    <row r="62" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D62" s="18" t="s">
+      <c r="M61" s="33"/>
+    </row>
+    <row r="62" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D62" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="E62" s="19"/>
-      <c r="F62" s="20" t="s">
+      <c r="E62" s="17"/>
+      <c r="F62" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="G62" s="21"/>
-      <c r="I62" s="22" t="s">
+      <c r="G62" s="19"/>
+      <c r="I62" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="J62" s="23"/>
-      <c r="L62" s="18" t="s">
+      <c r="J62" s="21"/>
+      <c r="L62" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="M62" s="21"/>
-    </row>
-    <row r="63" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D63" s="22"/>
-      <c r="E63" s="24"/>
-      <c r="F63" s="19"/>
-      <c r="G63" s="23"/>
-      <c r="I63" s="22"/>
-      <c r="J63" s="23"/>
-      <c r="L63" s="22"/>
-      <c r="M63" s="23"/>
-    </row>
-    <row r="64" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D64" s="22"/>
-      <c r="E64" s="24"/>
-      <c r="F64" s="19"/>
-      <c r="G64" s="21"/>
-      <c r="I64" s="22"/>
-      <c r="J64" s="23"/>
-      <c r="L64" s="22"/>
-      <c r="M64" s="23"/>
-    </row>
-    <row r="65" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D65" s="22"/>
-      <c r="E65" s="24"/>
-      <c r="F65" s="20" t="s">
+      <c r="M62" s="19"/>
+    </row>
+    <row r="63" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D63" s="20"/>
+      <c r="E63" s="22"/>
+      <c r="F63" s="17"/>
+      <c r="G63" s="21"/>
+      <c r="I63" s="20"/>
+      <c r="J63" s="21"/>
+      <c r="L63" s="20"/>
+      <c r="M63" s="21"/>
+    </row>
+    <row r="64" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D64" s="20"/>
+      <c r="E64" s="22"/>
+      <c r="F64" s="17"/>
+      <c r="G64" s="19"/>
+      <c r="I64" s="20"/>
+      <c r="J64" s="21"/>
+      <c r="L64" s="20"/>
+      <c r="M64" s="21"/>
+    </row>
+    <row r="65" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D65" s="20"/>
+      <c r="E65" s="22"/>
+      <c r="F65" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G65" s="21"/>
-      <c r="I65" s="18" t="s">
+      <c r="G65" s="19"/>
+      <c r="I65" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="J65" s="23"/>
-      <c r="L65" s="18" t="s">
+      <c r="J65" s="21"/>
+      <c r="L65" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="M65" s="23"/>
-    </row>
-    <row r="66" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D66" s="22"/>
-      <c r="E66" s="24"/>
-      <c r="F66" s="19" t="s">
+      <c r="M65" s="21"/>
+    </row>
+    <row r="66" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D66" s="20"/>
+      <c r="E66" s="22"/>
+      <c r="F66" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="G66" s="23">
+      <c r="G66" s="21">
         <v>1000000</v>
       </c>
-      <c r="I66" s="22" t="s">
+      <c r="I66" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="J66" s="23">
+      <c r="J66" s="21">
         <f>-G67</f>
         <v>-50000</v>
       </c>
-      <c r="L66" s="22"/>
-      <c r="M66" s="23"/>
-    </row>
-    <row r="67" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D67" s="25"/>
-      <c r="E67" s="26"/>
-      <c r="F67" s="27" t="s">
+      <c r="L66" s="20"/>
+      <c r="M66" s="21"/>
+    </row>
+    <row r="67" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D67" s="23"/>
+      <c r="E67" s="24"/>
+      <c r="F67" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="G67" s="28">
+      <c r="G67" s="26">
         <f>C57*C56</f>
         <v>50000</v>
       </c>
-      <c r="I67" s="29" t="s">
+      <c r="I67" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="J67" s="28">
+      <c r="J67" s="26">
         <f>J66</f>
         <v>-50000</v>
       </c>
-      <c r="L67" s="25"/>
-      <c r="M67" s="28"/>
-    </row>
-    <row r="68" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15"/>
-    <row r="69" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15"/>
-    <row r="70" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="B70" s="6" t="s">
+      <c r="L67" s="23"/>
+      <c r="M67" s="26"/>
+    </row>
+    <row r="68" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15"/>
+    <row r="69" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15"/>
+    <row r="70" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="B70" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="71" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15"/>
-    <row r="72" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D72" s="2" t="s">
+    <row r="71" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15"/>
+    <row r="72" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D72" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E72" s="2"/>
-      <c r="F72" s="2"/>
-      <c r="G72" s="2"/>
-      <c r="I72" s="2" t="s">
+      <c r="E72" s="32"/>
+      <c r="F72" s="32"/>
+      <c r="G72" s="32"/>
+      <c r="I72" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="J72" s="2"/>
-      <c r="L72" s="2" t="s">
+      <c r="J72" s="32"/>
+      <c r="L72" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="M72" s="2"/>
-    </row>
-    <row r="73" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D73" s="7" t="s">
+      <c r="M72" s="32"/>
+    </row>
+    <row r="73" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D73" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F73" s="8" t="s">
+      <c r="F73" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G73" s="9"/>
-      <c r="I73" s="10" t="s">
+      <c r="G73" s="7"/>
+      <c r="I73" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="J73" s="11"/>
-      <c r="L73" s="7" t="s">
+      <c r="J73" s="9"/>
+      <c r="L73" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M73" s="9"/>
-    </row>
-    <row r="74" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D74" s="10" t="s">
+      <c r="M73" s="7"/>
+    </row>
+    <row r="74" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D74" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E74" s="4">
+      <c r="E74" s="2">
         <f>+-C57*C56</f>
         <v>-50000</v>
       </c>
-      <c r="G74" s="11"/>
-      <c r="I74" s="10"/>
-      <c r="J74" s="11"/>
-      <c r="L74" s="10"/>
-      <c r="M74" s="11"/>
-    </row>
-    <row r="75" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D75" s="10"/>
-      <c r="E75" s="4"/>
-      <c r="G75" s="9"/>
-      <c r="I75" s="10"/>
-      <c r="J75" s="11"/>
-      <c r="L75" s="10"/>
-      <c r="M75" s="11"/>
-    </row>
-    <row r="76" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D76" s="10"/>
-      <c r="E76" s="4"/>
-      <c r="F76" s="8" t="s">
+      <c r="G74" s="9"/>
+      <c r="I74" s="8"/>
+      <c r="J74" s="9"/>
+      <c r="L74" s="8"/>
+      <c r="M74" s="9"/>
+    </row>
+    <row r="75" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D75" s="8"/>
+      <c r="E75" s="2"/>
+      <c r="G75" s="7"/>
+      <c r="I75" s="8"/>
+      <c r="J75" s="9"/>
+      <c r="L75" s="8"/>
+      <c r="M75" s="9"/>
+    </row>
+    <row r="76" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D76" s="8"/>
+      <c r="E76" s="2"/>
+      <c r="F76" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G76" s="9"/>
-      <c r="I76" s="7" t="s">
+      <c r="G76" s="7"/>
+      <c r="I76" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J76" s="11"/>
-      <c r="L76" s="7" t="s">
+      <c r="J76" s="9"/>
+      <c r="L76" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="M76" s="11"/>
-    </row>
-    <row r="77" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D77" s="10"/>
-      <c r="E77" s="4"/>
+      <c r="M76" s="9"/>
+    </row>
+    <row r="77" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D77" s="8"/>
+      <c r="E77" s="2"/>
       <c r="F77" t="s">
         <v>24</v>
       </c>
-      <c r="G77" s="11">
+      <c r="G77" s="9">
         <v>-1000000</v>
       </c>
-      <c r="I77" s="10" t="s">
+      <c r="I77" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="J77" s="11"/>
-      <c r="L77" s="10" t="s">
+      <c r="J77" s="9"/>
+      <c r="L77" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="M77" s="11">
+      <c r="M77" s="9">
         <f>+E74</f>
         <v>-50000</v>
       </c>
     </row>
-    <row r="78" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D78" s="10"/>
-      <c r="E78" s="4"/>
+    <row r="78" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D78" s="8"/>
+      <c r="E78" s="2"/>
       <c r="F78" t="s">
         <v>16</v>
       </c>
-      <c r="G78" s="11">
+      <c r="G78" s="9">
         <v>1000000</v>
       </c>
-      <c r="I78" s="16" t="s">
+      <c r="I78" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="J78" s="17"/>
-      <c r="L78" s="12"/>
-      <c r="M78" s="17"/>
-    </row>
-    <row r="79" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D79" s="12"/>
-      <c r="E79" s="13"/>
-      <c r="F79" s="14" t="s">
+      <c r="J78" s="15"/>
+      <c r="L78" s="10"/>
+      <c r="M78" s="15"/>
+    </row>
+    <row r="79" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D79" s="10"/>
+      <c r="E79" s="11"/>
+      <c r="F79" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="G79" s="17">
+      <c r="G79" s="15">
         <f>-C56*C57</f>
         <v>-50000</v>
       </c>
     </row>
-    <row r="80" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15"/>
-    <row r="81" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15"/>
-    <row r="82" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="B82" s="6" t="s">
+    <row r="80" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15"/>
+    <row r="81" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15"/>
+    <row r="82" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="B82" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="83" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15"/>
-    <row r="84" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D84" s="2" t="s">
+    <row r="83" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15"/>
+    <row r="84" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D84" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E84" s="2"/>
-      <c r="F84" s="2"/>
-      <c r="G84" s="2"/>
-      <c r="I84" s="2" t="s">
+      <c r="E84" s="32"/>
+      <c r="F84" s="32"/>
+      <c r="G84" s="32"/>
+      <c r="I84" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="J84" s="2"/>
-      <c r="L84" s="2" t="s">
+      <c r="J84" s="32"/>
+      <c r="L84" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="M84" s="2"/>
-    </row>
-    <row r="85" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D85" s="7" t="s">
+      <c r="M84" s="32"/>
+    </row>
+    <row r="85" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D85" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F85" s="8" t="s">
+      <c r="F85" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G85" s="9"/>
-      <c r="I85" s="10" t="s">
+      <c r="G85" s="7"/>
+      <c r="I85" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="J85" s="11"/>
-      <c r="L85" s="7" t="s">
+      <c r="J85" s="9"/>
+      <c r="L85" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M85" s="9"/>
-    </row>
-    <row r="86" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D86" s="10" t="s">
+      <c r="M85" s="7"/>
+    </row>
+    <row r="86" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D86" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E86" s="4"/>
-      <c r="G86" s="11"/>
-      <c r="I86" s="10"/>
-      <c r="J86" s="11"/>
-      <c r="L86" s="10"/>
-      <c r="M86" s="11"/>
-    </row>
-    <row r="87" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D87" s="10"/>
-      <c r="E87" s="4"/>
-      <c r="G87" s="9"/>
-      <c r="I87" s="10"/>
-      <c r="J87" s="11"/>
-      <c r="L87" s="10"/>
-      <c r="M87" s="11"/>
-    </row>
-    <row r="88" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D88" s="10"/>
-      <c r="E88" s="4"/>
-      <c r="F88" s="8" t="s">
+      <c r="E86" s="2"/>
+      <c r="G86" s="9"/>
+      <c r="I86" s="8"/>
+      <c r="J86" s="9"/>
+      <c r="L86" s="8"/>
+      <c r="M86" s="9"/>
+    </row>
+    <row r="87" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D87" s="8"/>
+      <c r="E87" s="2"/>
+      <c r="G87" s="7"/>
+      <c r="I87" s="8"/>
+      <c r="J87" s="9"/>
+      <c r="L87" s="8"/>
+      <c r="M87" s="9"/>
+    </row>
+    <row r="88" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D88" s="8"/>
+      <c r="E88" s="2"/>
+      <c r="F88" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G88" s="9"/>
-      <c r="I88" s="7" t="s">
+      <c r="G88" s="7"/>
+      <c r="I88" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J88" s="11"/>
-      <c r="L88" s="7" t="s">
+      <c r="J88" s="9"/>
+      <c r="L88" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="M88" s="11"/>
-    </row>
-    <row r="89" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D89" s="10"/>
-      <c r="E89" s="4"/>
-      <c r="G89" s="11"/>
-      <c r="I89" s="10" t="s">
+      <c r="M88" s="9"/>
+    </row>
+    <row r="89" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D89" s="8"/>
+      <c r="E89" s="2"/>
+      <c r="G89" s="9"/>
+      <c r="I89" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="J89" s="11">
+      <c r="J89" s="9">
         <f>-G90</f>
         <v>-100000</v>
       </c>
-      <c r="L89" s="10"/>
-      <c r="M89" s="11"/>
-    </row>
-    <row r="90" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15">
-      <c r="D90" s="12"/>
-      <c r="E90" s="13"/>
-      <c r="F90" s="14" t="s">
+      <c r="L89" s="8"/>
+      <c r="M89" s="9"/>
+    </row>
+    <row r="90" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="D90" s="10"/>
+      <c r="E90" s="11"/>
+      <c r="F90" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="G90" s="17">
+      <c r="G90" s="15">
         <f>D57*C56</f>
         <v>100000</v>
       </c>
-      <c r="I90" s="16" t="s">
+      <c r="I90" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="J90" s="17">
+      <c r="J90" s="15">
         <f>J89</f>
         <v>-100000</v>
       </c>
-      <c r="L90" s="12"/>
-      <c r="M90" s="17"/>
-    </row>
-    <row r="91" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15"/>
-    <row r="92" spans="2:13" ht="13" hidden="1" outlineLevel="1" x14ac:dyDescent="0.15"/>
-    <row r="93" spans="2:13" ht="15" collapsed="1" x14ac:dyDescent="0.15">
-      <c r="B93" s="6" t="s">
+      <c r="L90" s="10"/>
+      <c r="M90" s="15"/>
+    </row>
+    <row r="91" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15"/>
+    <row r="92" spans="2:13" ht="13" outlineLevel="1" x14ac:dyDescent="0.15"/>
+    <row r="93" spans="2:13" ht="15" x14ac:dyDescent="0.15">
+      <c r="B93" s="4" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="95" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D95" s="2" t="s">
+      <c r="D95" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E95" s="2"/>
-      <c r="F95" s="2"/>
-      <c r="G95" s="2"/>
-      <c r="I95" s="2" t="s">
+      <c r="E95" s="32"/>
+      <c r="F95" s="32"/>
+      <c r="G95" s="32"/>
+      <c r="I95" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="J95" s="2"/>
-      <c r="L95" s="2" t="s">
+      <c r="J95" s="32"/>
+      <c r="L95" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="M95" s="2"/>
+      <c r="M95" s="32"/>
     </row>
     <row r="96" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D96" s="7" t="s">
+      <c r="D96" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F96" s="8" t="s">
+      <c r="F96" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G96" s="9"/>
-      <c r="I96" s="10" t="s">
+      <c r="G96" s="7"/>
+      <c r="I96" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="J96" s="11"/>
-      <c r="L96" s="7" t="s">
+      <c r="J96" s="9"/>
+      <c r="L96" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M96" s="9"/>
+      <c r="M96" s="7"/>
     </row>
     <row r="97" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D97" s="10" t="s">
+      <c r="D97" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E97" s="4">
+      <c r="E97" s="2">
         <f>+E74</f>
         <v>-50000</v>
       </c>
-      <c r="G97" s="11"/>
-      <c r="I97" s="10"/>
-      <c r="J97" s="11"/>
-      <c r="L97" s="10"/>
-      <c r="M97" s="11"/>
+      <c r="G97" s="9"/>
+      <c r="I97" s="8"/>
+      <c r="J97" s="9"/>
+      <c r="L97" s="8"/>
+      <c r="M97" s="9"/>
     </row>
     <row r="98" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D98" s="10"/>
-      <c r="E98" s="4"/>
-      <c r="G98" s="9"/>
-      <c r="I98" s="10"/>
-      <c r="J98" s="11"/>
-      <c r="L98" s="10"/>
-      <c r="M98" s="11"/>
+      <c r="D98" s="8"/>
+      <c r="E98" s="2"/>
+      <c r="G98" s="7"/>
+      <c r="I98" s="8"/>
+      <c r="J98" s="9"/>
+      <c r="L98" s="8"/>
+      <c r="M98" s="9"/>
     </row>
     <row r="99" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D99" s="10"/>
-      <c r="E99" s="4"/>
-      <c r="F99" s="8" t="s">
+      <c r="D99" s="8"/>
+      <c r="E99" s="2"/>
+      <c r="F99" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G99" s="9"/>
-      <c r="I99" s="7" t="s">
+      <c r="G99" s="7"/>
+      <c r="I99" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J99" s="11"/>
-      <c r="L99" s="7" t="s">
+      <c r="J99" s="9"/>
+      <c r="L99" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="M99" s="11"/>
+      <c r="M99" s="9"/>
     </row>
     <row r="100" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D100" s="10"/>
-      <c r="E100" s="4"/>
+      <c r="D100" s="8"/>
+      <c r="E100" s="2"/>
       <c r="F100" t="s">
         <v>24</v>
       </c>
-      <c r="G100" s="11">
+      <c r="G100" s="9">
         <f>G77</f>
         <v>-1000000</v>
       </c>
-      <c r="I100" s="10" t="s">
+      <c r="I100" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="J100" s="11">
+      <c r="J100" s="9">
         <f>+J89</f>
         <v>-100000</v>
       </c>
-      <c r="L100" s="10" t="s">
+      <c r="L100" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="M100" s="11">
+      <c r="M100" s="9">
         <f>+E97</f>
         <v>-50000</v>
       </c>
     </row>
     <row r="101" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D101" s="10"/>
-      <c r="E101" s="4"/>
+      <c r="D101" s="8"/>
+      <c r="E101" s="2"/>
       <c r="F101" t="s">
         <v>16</v>
       </c>
-      <c r="G101" s="11">
+      <c r="G101" s="9">
         <f>+G78</f>
         <v>1000000</v>
       </c>
-      <c r="I101" s="16" t="s">
+      <c r="I101" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="J101" s="17">
+      <c r="J101" s="15">
         <f>J100</f>
         <v>-100000</v>
       </c>
-      <c r="L101" s="12"/>
-      <c r="M101" s="17"/>
+      <c r="L101" s="10"/>
+      <c r="M101" s="15"/>
     </row>
     <row r="102" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="D102" s="12"/>
-      <c r="E102" s="14"/>
-      <c r="F102" s="14" t="s">
+      <c r="D102" s="10"/>
+      <c r="E102" s="12"/>
+      <c r="F102" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="G102" s="17">
+      <c r="G102" s="15">
         <f>+G79+G90</f>
         <v>50000</v>
       </c>
     </row>
     <row r="105" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="B105" s="30" t="s">
+      <c r="B105" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="C105" s="30"/>
-      <c r="D105" s="30" t="s">
+      <c r="C105" s="28"/>
+      <c r="D105" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="E105" s="30"/>
-      <c r="F105" s="30" t="s">
+      <c r="E105" s="28"/>
+      <c r="F105" s="28" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="106" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="B106" s="3" t="s">
+      <c r="B106" s="1" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="107" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="B107" s="3"/>
+      <c r="B107" s="1"/>
       <c r="C107" t="s">
         <v>38</v>
       </c>
       <c r="D107" t="s">
         <v>39</v>
       </c>
-      <c r="F107" s="31" t="s">
+      <c r="F107" s="29" t="s">
         <v>40</v>
       </c>
       <c r="I107" t="s">
@@ -1810,40 +1810,40 @@
       </c>
     </row>
     <row r="108" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="B108" s="3"/>
+      <c r="B108" s="1"/>
       <c r="C108" t="s">
         <v>42</v>
       </c>
       <c r="D108" t="s">
         <v>39</v>
       </c>
-      <c r="F108" s="31" t="s">
+      <c r="F108" s="29" t="s">
         <v>40</v>
       </c>
       <c r="H108" t="s">
         <v>43</v>
       </c>
-      <c r="I108" s="4">
+      <c r="I108" s="2">
         <v>5000000</v>
       </c>
     </row>
     <row r="109" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="B109" s="3" t="s">
+      <c r="B109" s="1" t="s">
         <v>44</v>
       </c>
       <c r="H109" t="s">
         <v>45</v>
       </c>
-      <c r="I109" s="4">
+      <c r="I109" s="2">
         <v>4000000</v>
       </c>
     </row>
     <row r="110" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="B110" s="3"/>
+      <c r="B110" s="1"/>
       <c r="C110" t="s">
         <v>46</v>
       </c>
-      <c r="D110" s="31" t="s">
+      <c r="D110" s="29" t="s">
         <v>40</v>
       </c>
       <c r="F110" t="s">
@@ -1852,22 +1852,22 @@
       <c r="H110" t="s">
         <v>47</v>
       </c>
-      <c r="I110" s="4">
+      <c r="I110" s="2">
         <v>1000000</v>
       </c>
     </row>
     <row r="111" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="B111" s="3" t="s">
+      <c r="B111" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D111" s="31"/>
+      <c r="D111" s="29"/>
     </row>
     <row r="112" spans="2:13" ht="13" x14ac:dyDescent="0.15">
-      <c r="B112" s="3"/>
+      <c r="B112" s="1"/>
       <c r="C112" t="s">
         <v>49</v>
       </c>
-      <c r="D112" s="31" t="s">
+      <c r="D112" s="29" t="s">
         <v>40</v>
       </c>
       <c r="F112" t="s">
@@ -1875,14 +1875,14 @@
       </c>
     </row>
     <row r="113" spans="2:11" ht="13" x14ac:dyDescent="0.15">
-      <c r="H113" s="30"/>
-      <c r="I113" s="30" t="s">
+      <c r="H113" s="28"/>
+      <c r="I113" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="J113" s="30" t="s">
+      <c r="J113" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="K113" s="30" t="s">
+      <c r="K113" s="28" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1894,11 +1894,11 @@
         <f>I109/I108</f>
         <v>0.8</v>
       </c>
-      <c r="J114" s="32">
+      <c r="J114" s="30">
         <f>(I109+G50+G51)/(I108-E47)</f>
         <v>0.48760330578512395</v>
       </c>
-      <c r="K114" s="32">
+      <c r="K114" s="30">
         <f>(I109+G102)/(I108+E97)</f>
         <v>0.81818181818181823</v>
       </c>
@@ -1925,30 +1925,30 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="D37:G37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="D45:G45"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="L45:M45"/>
+    <mergeCell ref="D61:G61"/>
+    <mergeCell ref="I61:J61"/>
+    <mergeCell ref="L61:M61"/>
+    <mergeCell ref="D72:G72"/>
+    <mergeCell ref="I72:J72"/>
+    <mergeCell ref="L72:M72"/>
     <mergeCell ref="D84:G84"/>
     <mergeCell ref="I84:J84"/>
     <mergeCell ref="L84:M84"/>
     <mergeCell ref="D95:G95"/>
     <mergeCell ref="I95:J95"/>
     <mergeCell ref="L95:M95"/>
-    <mergeCell ref="D61:G61"/>
-    <mergeCell ref="I61:J61"/>
-    <mergeCell ref="L61:M61"/>
-    <mergeCell ref="D72:G72"/>
-    <mergeCell ref="I72:J72"/>
-    <mergeCell ref="L72:M72"/>
-    <mergeCell ref="D37:G37"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="L37:M37"/>
-    <mergeCell ref="D45:G45"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="L45:M45"/>
-    <mergeCell ref="D9:G9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="D20:G20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="L20:M20"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1973,214 +1973,214 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="4" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="I4" s="2" t="s">
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="I4" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="J4" s="2"/>
-      <c r="L4" s="2" t="s">
+      <c r="J4" s="32"/>
+      <c r="L4" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="M4" s="2"/>
+      <c r="M4" s="32"/>
     </row>
     <row r="5" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="9"/>
-      <c r="I5" s="10" t="s">
+      <c r="G5" s="7"/>
+      <c r="I5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="11"/>
-      <c r="L5" s="7" t="s">
+      <c r="J5" s="9"/>
+      <c r="L5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M5" s="9"/>
+      <c r="M5" s="7"/>
     </row>
     <row r="6" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="2">
         <v>1000000</v>
       </c>
       <c r="F6" t="s">
         <v>57</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="9">
         <v>1000000</v>
       </c>
-      <c r="I6" s="10"/>
-      <c r="J6" s="11"/>
-      <c r="L6" s="10" t="s">
+      <c r="I6" s="8"/>
+      <c r="J6" s="9"/>
+      <c r="L6" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="M6" s="11">
+      <c r="M6" s="9">
         <f>+E6</f>
         <v>1000000</v>
       </c>
     </row>
     <row r="7" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D7" s="10"/>
-      <c r="E7" s="4"/>
-      <c r="G7" s="9"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="11"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="11"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="2"/>
+      <c r="G7" s="7"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="9"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="9"/>
     </row>
     <row r="8" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D8" s="10"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="8" t="s">
+      <c r="D8" s="8"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="9"/>
-      <c r="I8" s="7" t="s">
+      <c r="G8" s="7"/>
+      <c r="I8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="11"/>
-      <c r="L8" s="7" t="s">
+      <c r="J8" s="9"/>
+      <c r="L8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="M8" s="11"/>
+      <c r="M8" s="9"/>
     </row>
     <row r="9" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D9" s="10"/>
-      <c r="E9" s="4"/>
-      <c r="G9" s="11"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="11"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="11"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="2"/>
+      <c r="G9" s="9"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="9"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="9"/>
     </row>
     <row r="10" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D10" s="12"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="15"/>
-      <c r="I10" s="16" t="s">
+      <c r="D10" s="10"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="13"/>
+      <c r="I10" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="J10" s="17"/>
-      <c r="L10" s="12"/>
-      <c r="M10" s="17"/>
+      <c r="J10" s="15"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="15"/>
     </row>
     <row r="13" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="1" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="15" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="I15" s="2" t="s">
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="32"/>
+      <c r="I15" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="J15" s="2"/>
-      <c r="L15" s="2" t="s">
+      <c r="J15" s="32"/>
+      <c r="L15" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="M15" s="2"/>
+      <c r="M15" s="32"/>
     </row>
     <row r="16" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G16" s="9"/>
-      <c r="I16" s="10" t="s">
+      <c r="G16" s="7"/>
+      <c r="I16" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="J16" s="11"/>
-      <c r="L16" s="7" t="s">
+      <c r="J16" s="9"/>
+      <c r="L16" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M16" s="9"/>
+      <c r="M16" s="7"/>
     </row>
     <row r="17" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="2">
         <v>-300000</v>
       </c>
       <c r="F17" t="s">
         <v>60</v>
       </c>
-      <c r="G17" s="11">
+      <c r="G17" s="9">
         <v>-300000</v>
       </c>
-      <c r="I17" s="10"/>
-      <c r="J17" s="11"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="9"/>
     </row>
     <row r="18" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D18" s="10"/>
-      <c r="E18" s="4"/>
-      <c r="G18" s="9"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="11"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="11"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="2"/>
+      <c r="G18" s="7"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="9"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="9"/>
     </row>
     <row r="19" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D19" s="10"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="8" t="s">
+      <c r="D19" s="8"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G19" s="9"/>
-      <c r="I19" s="7" t="s">
+      <c r="G19" s="7"/>
+      <c r="I19" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J19" s="11"/>
-      <c r="L19" s="7" t="s">
+      <c r="J19" s="9"/>
+      <c r="L19" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="M19" s="11"/>
+      <c r="M19" s="9"/>
     </row>
     <row r="20" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D20" s="10"/>
-      <c r="E20" s="4"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="11"/>
-      <c r="L20" s="10" t="s">
+      <c r="D20" s="8"/>
+      <c r="E20" s="2"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="9"/>
+      <c r="L20" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="M20" s="11">
+      <c r="M20" s="9">
         <v>-300000</v>
       </c>
     </row>
     <row r="21" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D21" s="12"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="15"/>
-      <c r="I21" s="16" t="s">
+      <c r="D21" s="10"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="13"/>
+      <c r="I21" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="J21" s="17"/>
-      <c r="L21" s="12"/>
-      <c r="M21" s="17"/>
+      <c r="J21" s="15"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="15"/>
     </row>
     <row r="25" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B25" t="s">
@@ -2193,7 +2193,7 @@
       </c>
     </row>
     <row r="27" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B27" s="33"/>
+      <c r="B27" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
minor updates in topic 2
</commit_message>
<xml_diff>
--- a/topic_2_img/Topic 2 Sol.xlsx
+++ b/topic_2_img/Topic 2 Sol.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Data/Github/lecture_financial_statements_analysis/topic_2_img/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A805BADB-298C-4C4F-ACCF-D1AF02E91AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C59699E-A60F-5242-85FF-219DECF0E3A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-35560" yWindow="2040" windowWidth="36060" windowHeight="20640" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-33720" yWindow="2040" windowWidth="33720" windowHeight="19200" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_loan" sheetId="1" r:id="rId1"/>
@@ -1925,30 +1925,30 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="D84:G84"/>
+    <mergeCell ref="I84:J84"/>
+    <mergeCell ref="L84:M84"/>
+    <mergeCell ref="D95:G95"/>
+    <mergeCell ref="I95:J95"/>
+    <mergeCell ref="L95:M95"/>
+    <mergeCell ref="D61:G61"/>
+    <mergeCell ref="I61:J61"/>
+    <mergeCell ref="L61:M61"/>
+    <mergeCell ref="D72:G72"/>
+    <mergeCell ref="I72:J72"/>
+    <mergeCell ref="L72:M72"/>
+    <mergeCell ref="D37:G37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="D45:G45"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="L45:M45"/>
     <mergeCell ref="D9:G9"/>
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="D20:G20"/>
     <mergeCell ref="I20:J20"/>
     <mergeCell ref="L20:M20"/>
-    <mergeCell ref="D37:G37"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="L37:M37"/>
-    <mergeCell ref="D45:G45"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="L45:M45"/>
-    <mergeCell ref="D61:G61"/>
-    <mergeCell ref="I61:J61"/>
-    <mergeCell ref="L61:M61"/>
-    <mergeCell ref="D72:G72"/>
-    <mergeCell ref="I72:J72"/>
-    <mergeCell ref="L72:M72"/>
-    <mergeCell ref="D84:G84"/>
-    <mergeCell ref="I84:J84"/>
-    <mergeCell ref="L84:M84"/>
-    <mergeCell ref="D95:G95"/>
-    <mergeCell ref="I95:J95"/>
-    <mergeCell ref="L95:M95"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
topic 2  change excel
</commit_message>
<xml_diff>
--- a/topic_2_img/Topic 2 Sol.xlsx
+++ b/topic_2_img/Topic 2 Sol.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Data/Github/lecture_financial_statements_analysis/topic_2_img/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C59699E-A60F-5242-85FF-219DECF0E3A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D055CCC7-8B14-5B42-A4F7-60108B7DE183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-33720" yWindow="2040" windowWidth="33720" windowHeight="19200" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="66">
   <si>
     <t>Part 1: Borrowing $1,000,000 from a bank at a 5% interest rate:</t>
   </si>
@@ -219,9 +219,6 @@
     <t>worse</t>
   </si>
   <si>
-    <t>better</t>
-  </si>
-  <si>
     <t>Hypothetical situation</t>
   </si>
   <si>
@@ -286,6 +283,18 @@
   </si>
   <si>
     <t>b) what if the capital increase is done via issuing 1.000 new shares to the market?</t>
+  </si>
+  <si>
+    <t>better (keep cash + lt debt)</t>
+  </si>
+  <si>
+    <t>better (keep cash)</t>
+  </si>
+  <si>
+    <t>better (no debt)</t>
+  </si>
+  <si>
+    <t>better (no interest expenses)</t>
   </si>
 </sst>
 </file>
@@ -1803,25 +1812,25 @@
         <v>39</v>
       </c>
       <c r="F107" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="I107" t="s">
         <v>40</v>
-      </c>
-      <c r="I107" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="108" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B108" s="1"/>
       <c r="C108" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D108" t="s">
         <v>39</v>
       </c>
       <c r="F108" s="29" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="H108" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I108" s="2">
         <v>5000000</v>
@@ -1829,10 +1838,10 @@
     </row>
     <row r="109" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B109" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H109" t="s">
         <v>44</v>
-      </c>
-      <c r="H109" t="s">
-        <v>45</v>
       </c>
       <c r="I109" s="2">
         <v>4000000</v>
@@ -1841,16 +1850,16 @@
     <row r="110" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B110" s="1"/>
       <c r="C110" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D110" s="29" t="s">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="F110" t="s">
         <v>39</v>
       </c>
       <c r="H110" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I110" s="2">
         <v>1000000</v>
@@ -1858,17 +1867,17 @@
     </row>
     <row r="111" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B111" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D111" s="29"/>
     </row>
     <row r="112" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B112" s="1"/>
       <c r="C112" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D112" s="29" t="s">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="F112" t="s">
         <v>39</v>
@@ -1877,7 +1886,7 @@
     <row r="113" spans="2:11" ht="13" x14ac:dyDescent="0.15">
       <c r="H113" s="28"/>
       <c r="I113" s="28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J113" s="28" t="s">
         <v>35</v>
@@ -1888,7 +1897,7 @@
     </row>
     <row r="114" spans="2:11" ht="13" x14ac:dyDescent="0.15">
       <c r="H114" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I114">
         <f>I109/I108</f>
@@ -1905,50 +1914,50 @@
     </row>
     <row r="116" spans="2:11" ht="13" x14ac:dyDescent="0.15">
       <c r="B116" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="117" spans="2:11" ht="13" x14ac:dyDescent="0.15">
       <c r="B117" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="118" spans="2:11" ht="13" x14ac:dyDescent="0.15">
       <c r="B118" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="119" spans="2:11" ht="13" x14ac:dyDescent="0.15">
       <c r="B119" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="D37:G37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="D45:G45"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="L45:M45"/>
+    <mergeCell ref="D61:G61"/>
+    <mergeCell ref="I61:J61"/>
+    <mergeCell ref="L61:M61"/>
+    <mergeCell ref="D72:G72"/>
+    <mergeCell ref="I72:J72"/>
+    <mergeCell ref="L72:M72"/>
     <mergeCell ref="D84:G84"/>
     <mergeCell ref="I84:J84"/>
     <mergeCell ref="L84:M84"/>
     <mergeCell ref="D95:G95"/>
     <mergeCell ref="I95:J95"/>
     <mergeCell ref="L95:M95"/>
-    <mergeCell ref="D61:G61"/>
-    <mergeCell ref="I61:J61"/>
-    <mergeCell ref="L61:M61"/>
-    <mergeCell ref="D72:G72"/>
-    <mergeCell ref="I72:J72"/>
-    <mergeCell ref="L72:M72"/>
-    <mergeCell ref="D37:G37"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="L37:M37"/>
-    <mergeCell ref="D45:G45"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="L45:M45"/>
-    <mergeCell ref="D9:G9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="D20:G20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="L20:M20"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1974,7 +1983,7 @@
   <sheetData>
     <row r="2" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B2" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -2018,7 +2027,7 @@
         <v>1000000</v>
       </c>
       <c r="F6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G6" s="9">
         <v>1000000</v>
@@ -2026,7 +2035,7 @@
       <c r="I6" s="8"/>
       <c r="J6" s="9"/>
       <c r="L6" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="M6" s="9">
         <f>+E6</f>
@@ -2081,7 +2090,7 @@
     </row>
     <row r="13" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B13" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -2125,7 +2134,7 @@
         <v>-300000</v>
       </c>
       <c r="F17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G17" s="9">
         <v>-300000</v>
@@ -2164,7 +2173,7 @@
       <c r="I20" s="8"/>
       <c r="J20" s="9"/>
       <c r="L20" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="M20" s="9">
         <v>-300000</v>
@@ -2184,12 +2193,12 @@
     </row>
     <row r="25" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B26" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
topic 2, last corrections and deleted old figures
</commit_message>
<xml_diff>
--- a/topic_2_img/Topic 2 Sol.xlsx
+++ b/topic_2_img/Topic 2 Sol.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Data/Github/lecture_financial_statements_analysis/topic_2_img/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D055CCC7-8B14-5B42-A4F7-60108B7DE183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53EF97B8-DD70-FB48-AEF5-6799DC6F6AD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-33720" yWindow="2040" windowWidth="33720" windowHeight="19200" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-33720" yWindow="2040" windowWidth="33720" windowHeight="19200" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_loan" sheetId="1" r:id="rId1"/>
@@ -267,9 +267,6 @@
     <t>Accounting event 1: capital increase</t>
   </si>
   <si>
-    <t>Capital Share</t>
-  </si>
-  <si>
     <t>Financing</t>
   </si>
   <si>
@@ -279,12 +276,6 @@
     <t>Retained earnings</t>
   </si>
   <si>
-    <t>a) What if dividends are announced that day but not paid yet?</t>
-  </si>
-  <si>
-    <t>b) what if the capital increase is done via issuing 1.000 new shares to the market?</t>
-  </si>
-  <si>
     <t>better (keep cash + lt debt)</t>
   </si>
   <si>
@@ -295,6 +286,15 @@
   </si>
   <si>
     <t>better (no interest expenses)</t>
+  </si>
+  <si>
+    <t>Share Capital</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> what if the capital increase is done via issuing 1.000 new shares to the market?</t>
+  </si>
+  <si>
+    <t>What if dividends are announced that day but will be paid in 60 days?</t>
   </si>
 </sst>
 </file>
@@ -1812,7 +1812,7 @@
         <v>39</v>
       </c>
       <c r="F107" s="29" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I107" t="s">
         <v>40</v>
@@ -1827,7 +1827,7 @@
         <v>39</v>
       </c>
       <c r="F108" s="29" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="H108" t="s">
         <v>42</v>
@@ -1853,7 +1853,7 @@
         <v>45</v>
       </c>
       <c r="D110" s="29" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F110" t="s">
         <v>39</v>
@@ -1877,7 +1877,7 @@
         <v>48</v>
       </c>
       <c r="D112" s="29" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F112" t="s">
         <v>39</v>
@@ -1934,30 +1934,30 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="D84:G84"/>
+    <mergeCell ref="I84:J84"/>
+    <mergeCell ref="L84:M84"/>
+    <mergeCell ref="D95:G95"/>
+    <mergeCell ref="I95:J95"/>
+    <mergeCell ref="L95:M95"/>
+    <mergeCell ref="D61:G61"/>
+    <mergeCell ref="I61:J61"/>
+    <mergeCell ref="L61:M61"/>
+    <mergeCell ref="D72:G72"/>
+    <mergeCell ref="I72:J72"/>
+    <mergeCell ref="L72:M72"/>
+    <mergeCell ref="D37:G37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="D45:G45"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="L45:M45"/>
     <mergeCell ref="D9:G9"/>
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="D20:G20"/>
     <mergeCell ref="I20:J20"/>
     <mergeCell ref="L20:M20"/>
-    <mergeCell ref="D37:G37"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="L37:M37"/>
-    <mergeCell ref="D45:G45"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="L45:M45"/>
-    <mergeCell ref="D61:G61"/>
-    <mergeCell ref="I61:J61"/>
-    <mergeCell ref="L61:M61"/>
-    <mergeCell ref="D72:G72"/>
-    <mergeCell ref="I72:J72"/>
-    <mergeCell ref="L72:M72"/>
-    <mergeCell ref="D84:G84"/>
-    <mergeCell ref="I84:J84"/>
-    <mergeCell ref="L84:M84"/>
-    <mergeCell ref="D95:G95"/>
-    <mergeCell ref="I95:J95"/>
-    <mergeCell ref="L95:M95"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2027,7 +2027,7 @@
         <v>1000000</v>
       </c>
       <c r="F6" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="G6" s="9">
         <v>1000000</v>
@@ -2035,7 +2035,7 @@
       <c r="I6" s="8"/>
       <c r="J6" s="9"/>
       <c r="L6" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M6" s="9">
         <f>+E6</f>
@@ -2088,9 +2088,14 @@
       <c r="L10" s="10"/>
       <c r="M10" s="15"/>
     </row>
+    <row r="11" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B11" t="s">
+        <v>64</v>
+      </c>
+    </row>
     <row r="13" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B13" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -2134,7 +2139,7 @@
         <v>-300000</v>
       </c>
       <c r="F17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G17" s="9">
         <v>-300000</v>
@@ -2173,7 +2178,7 @@
       <c r="I20" s="8"/>
       <c r="J20" s="9"/>
       <c r="L20" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M20" s="9">
         <v>-300000</v>
@@ -2193,12 +2198,7 @@
     </row>
     <row r="25" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B25" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="26" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B26" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>